<commit_message>
adding slides from data culture workshop
</commit_message>
<xml_diff>
--- a/On-the-job and self-study.xlsx
+++ b/On-the-job and self-study.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DE Apprenticeship\Learning-Journal\Learning-Journal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80FD765B-1848-4AB2-904F-9CE8FEF7996F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C36BDE21-78A7-4BFD-A0CD-7F4FC2016AA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{87251D64-A23B-4DC4-BF2E-D68309477306}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{87251D64-A23B-4DC4-BF2E-D68309477306}"/>
   </bookViews>
   <sheets>
     <sheet name="Log" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="33">
   <si>
     <t>On-the-job and self-guided learning hours log.</t>
   </si>
@@ -144,6 +144,9 @@
   </si>
   <si>
     <t>10.03.2025</t>
+  </si>
+  <si>
+    <t>18.03.2025</t>
   </si>
 </sst>
 </file>
@@ -831,7 +834,7 @@
       <c r="C6" s="17"/>
       <c r="D6" s="15">
         <f>SUM(B9:E51)</f>
-        <v>16.5</v>
+        <v>17.5</v>
       </c>
       <c r="E6" s="13"/>
       <c r="F6" s="17" t="s">
@@ -1073,10 +1076,14 @@
       <c r="H21" s="10"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="5"/>
+      <c r="A22" s="5" t="s">
+        <v>32</v>
+      </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
+      <c r="D22" s="7">
+        <v>1</v>
+      </c>
       <c r="E22" s="7"/>
       <c r="F22" s="9"/>
       <c r="G22" s="9"/>

</xml_diff>